<commit_message>
Show the player's own rank on the leaderboard, list the top 50, and keep the podium still
The board now lists 50 cooks. The player's own row is brown with a YOU chip;
when they are outside the top 50 it stays pinned under the list with their real
rank, which get_leaderboard.php now returns for ?me=<id> using the board's own
ordering. Inside the top 50 the row pins to the bottom until it is scrolled to,
then to the top once scrolled past. Only the ranks scroll; the header and podium
stay put. Older app versions get the same reply as before.
</commit_message>
<xml_diff>
--- a/docs/testing/KusinaKode_Timetable.xlsx
+++ b/docs/testing/KusinaKode_Timetable.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Progress Table" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progress" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Integration and Unit" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration and Unit" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -179,7 +179,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -191,11 +191,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1089,7 +1089,7 @@
     </row>
     <row r="14">
       <c r="B14" s="11" t="n"/>
-      <c r="C14" s="12" t="n"/>
+      <c r="C14" s="8" t="n"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Points calculation on round completion</t>
@@ -1298,8 +1298,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="12" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="13" t="n"/>
       <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Phase 1: event trigger + AES-256 encrypt + SHA-256 hash</t>
@@ -1718,8 +1718,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="8" t="n"/>
+      <c r="B32" s="12" t="n"/>
+      <c r="C32" s="13" t="n"/>
       <c r="D32" s="4" t="inlineStr">
         <is>
           <t>User CRUD and search</t>
@@ -1842,8 +1842,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="13" t="n"/>
-      <c r="C36" s="8" t="n"/>
+      <c r="B36" s="12" t="n"/>
+      <c r="C36" s="13" t="n"/>
       <c r="D36" s="4" t="inlineStr">
         <is>
           <t>Login and sign-up (mobile)</t>
@@ -2049,7 +2049,7 @@
     </row>
     <row r="42">
       <c r="B42" s="6" t="n"/>
-      <c r="C42" s="8" t="n"/>
+      <c r="C42" s="13" t="n"/>
       <c r="D42" s="4" t="inlineStr">
         <is>
           <t>Azure VM (PHP REST API + blockchain node)</t>
@@ -2277,7 +2277,7 @@
     </row>
     <row r="50">
       <c r="B50" s="6" t="n"/>
-      <c r="C50" s="8" t="n"/>
+      <c r="C50" s="13" t="n"/>
       <c r="D50" s="4" t="inlineStr">
         <is>
           <t>Unit tests per module (5-module breakdown)</t>
@@ -2648,7 +2648,7 @@
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>Built 2026-08-25 (Mau): KusinaNotifications with Rewards and Reminders channels, POST_NOTIFICATIONS runtime request, a notification when a badge finishes minting, and a daily-claim nudge on app open. NOT DONE: reminders while the app is closed (streak nudge, end-of-day daily warning) - those need WorkManager, which was deliberately not added. Verified permission prompt on emulator. In-app Notifications screen added behind the Home header bell - claimable rewards plus every on-chain reward with its TxHash, since system notifications vanish once dismissed. Bell count (D-41, 2026-09-16): daily claim is two waiting rows (KK + palayok), so the badge matches WAITING FOR YOU. Inbox (2026-09-16): minted title drops the bang and status is title-cased (Confirmed); Mark all read / Select / Archived sit on the right. On-chain list is newest-first (2026-09-17). Ledger ticket (D-43): report is a button, details are required, Done hides while filing. Junk like aaa is rejected (D-45: 12+ characters in the player's own words). Daily inbox title is Daily 2026-09-17; Recorded converts UTC to the phone's local time. Island complete (2026-09-17, D-46): CLAIMED chip plus waiting/claimed notifications, same as Daily Login. Palayok free spin (D-47, 2026-09-17): daily claim banks the spin; a claimed day missing one is repaired on the next pantry snapshot. Inbox (D-48, 2026-09-17): resume refreshes so a claimed daily moves to On-Chain Activity; Daily palayok spin stays in Waiting until the wheel is turned. After the wheel (D-49, 2026-09-17): pantry/spin.php writes a palayok_spin receipt (0 KK) so On-Chain Activity lists Daily login claim then Daily palayok spin. Waiting titles match those two names. Inbox chrome (2026-09-17): parchment cards matching Settings, one box per row, no circular wells.</t>
+          <t>Built 2026-08-25 (Mau): KusinaNotifications with Rewards and Reminders channels, POST_NOTIFICATIONS runtime request, a notification when a badge finishes minting, and a daily-claim nudge on app open. NOT DONE: reminders while the app is closed (streak nudge, end-of-day daily warning) - those need WorkManager, which was deliberately not added. Verified permission prompt on emulator. In-app Notifications screen added behind the Home header bell - claimable rewards plus every on-chain reward with its TxHash, since system notifications vanish once dismissed. Bell count (D-41, 2026-09-16): daily claim is two waiting rows (KK + palayok), so the badge matches WAITING FOR YOU. Inbox (2026-09-16): minted title drops the bang and status is title-cased (Confirmed); Mark all read / Select / Archived sit on the right. On-chain list is newest-first (2026-09-17). Ledger ticket (D-43): report is a button, details are required, Done hides while filing. Junk like aaa is rejected (D-45: 12+ characters in the player's own words). Daily inbox title is Daily 2026-09-17; Recorded converts UTC to the phone's local time. Island complete (2026-09-17, D-46): CLAIMED chip plus waiting/claimed notifications, same as Daily Login. Palayok free spin (D-47, 2026-09-17): daily claim banks the spin; a claimed day missing one is repaired on the next pantry snapshot. Inbox (D-48, 2026-09-17): resume refreshes so a claimed daily moves to On-Chain Activity; Daily palayok spin stays in Waiting until the wheel is turned. After the wheel (D-49, 2026-09-17): pantry/spin.php writes a palayok_spin receipt (0 KK) so On-Chain Activity lists Daily login claim then Daily palayok spin. Waiting titles match those two names. Inbox chrome (2026-09-17): parchment cards matching Settings, one box per row, no circular wells. Empty inbox (2026-10-11): a tab with nothing to claim or show uses the same centered message as KK Transaction, with the brown bell and no note card.</t>
         </is>
       </c>
     </row>
@@ -2758,8 +2758,8 @@
       </c>
     </row>
     <row r="64">
-      <c r="B64" s="14" t="n"/>
-      <c r="C64" s="14" t="n"/>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="6" t="n"/>
       <c r="D64" s="4" t="inlineStr">
         <is>
           <t>Downloadable badge certificate (PDF) on claim</t>
@@ -2788,15 +2788,142 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="B65" s="6" t="n"/>
+      <c r="C65" s="6" t="n"/>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Palayok open one or all</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F65" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr"/>
+      <c r="H65" s="4" t="inlineStr"/>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>Alyssa</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>A single waiting palayok offers Draw 1 only. Open all appears when two or more are waiting. When the pot opens it stays in the middle, and the ingredient rises out of it and floats just above. Checked on the emulator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Shelf ingredient trading card</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F66" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr"/>
+      <c r="H66" s="4" t="inlineStr"/>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>Alyssa</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>Tapping an ingredient already on the shelf opens the collectible card, the same size as the palayok card. The category, such as Vegetable, is one brown with a light edge so it stays readable on every frame, including Legendary, and it sits above the description. The quantity, such as 1 ON THE SHELF, is near-black on pale cards and light on the blue card. A palayok reveal still says INGREDIENT UNLOCKED and SHELVED IN YOUR PANTRY. The name banner shrinks until the full title fits, including a closing parenthesis. Checked on the emulator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="6" t="n"/>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Pantry duplicate sell quantity</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F67" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr"/>
+      <c r="H67" s="4" t="inlineStr"/>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>Alyssa</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>KODEX Pantry Sell on a stack of 2 or more opens a chooser from 1 to the owned count, shows the KK for that count, and sells only the chosen number. The chooser is a terracotta slider with minus on the left and plus on the right, on the same parchment card. A single copy still confirms a sale of 1. The older pantry shelf uses the same chooser. Unit-tested the count clamp. Alyssa checked the chooser on the emulator: terracotta track and knob, and small Sell-style minus and plus with no bottom shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="14" t="n"/>
+      <c r="C68" s="14" t="n"/>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Leaderboard shows your own rank</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Mobile / Backend</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr"/>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>Mau</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>Kusina Masters lists the top 50. The player's own row is brown with a YOU chip; outside the top 50 it stays pinned under the list with the real rank (get_leaderboard.php?me= returns it, using the board's own ordering). Inside the top 50 it pins to the bottom until scrolled to, then to the top once scrolled past. The header and podium no longer scroll. Older app versions get the same reply as before. Unit-tested in LeaderboardViewModelTest; checked on the emulator at rank #39 and #32.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="C20:C64"/>
-    <mergeCell ref="B2:B57"/>
-    <mergeCell ref="B20:B64"/>
-    <mergeCell ref="B14:B61"/>
+  <mergeCells count="6">
+    <mergeCell ref="C9:C66"/>
+    <mergeCell ref="B2:B66"/>
+    <mergeCell ref="A2:A68"/>
     <mergeCell ref="C2:C57"/>
-    <mergeCell ref="A2:A64"/>
-    <mergeCell ref="C14:C61"/>
+    <mergeCell ref="C14:C68"/>
+    <mergeCell ref="B14:B68"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2867,23 +2994,23 @@
     </row>
     <row r="6">
       <c r="A6" s="17">
-        <f>COUNTA('Progress Table'!$F$2:$F$64)</f>
+        <f>COUNTA('Progress Table'!$F$2:$F$68)</f>
         <v/>
       </c>
       <c r="B6" s="17">
-        <f>COUNTIF('Progress Table'!$F$2:$F$64,"OK")</f>
+        <f>COUNTIF('Progress Table'!$F$2:$F$68,"OK")</f>
         <v/>
       </c>
       <c r="C6" s="17">
-        <f>COUNTIF('Progress Table'!$F$2:$F$64,"In Progress")</f>
+        <f>COUNTIF('Progress Table'!$F$2:$F$68,"In Progress")</f>
         <v/>
       </c>
       <c r="D6" s="17">
-        <f>COUNTIF('Progress Table'!$F$2:$F$64,"Not Started")</f>
+        <f>COUNTIF('Progress Table'!$F$2:$F$68,"Not Started")</f>
         <v/>
       </c>
       <c r="E6" s="17">
-        <f>COUNTIF('Progress Table'!$F$2:$F$64,"Scope Change")</f>
+        <f>COUNTIF('Progress Table'!$F$2:$F$68,"Scope Change")</f>
         <v/>
       </c>
       <c r="F6" s="18">
@@ -2959,11 +3086,11 @@
         </is>
       </c>
       <c r="C10" s="19">
-        <f>COUNTA('Progress Table'!$F$9:$F$13)</f>
+        <f>COUNTA('Progress Table'!$F$9:$F$66)</f>
         <v/>
       </c>
       <c r="D10" s="19">
-        <f>COUNTIF('Progress Table'!$F$9:$F$13,"OK")</f>
+        <f>COUNTIF('Progress Table'!$F$9:$F$66,"OK")</f>
         <v/>
       </c>
       <c r="E10" s="20">
@@ -2985,11 +3112,11 @@
         </is>
       </c>
       <c r="C11" s="19">
-        <f>COUNTA('Progress Table'!$F$14:$F$61)</f>
+        <f>COUNTA('Progress Table'!$F$14:$F$68)</f>
         <v/>
       </c>
       <c r="D11" s="19">
-        <f>COUNTIF('Progress Table'!$F$14:$F$61,"OK")</f>
+        <f>COUNTIF('Progress Table'!$F$14:$F$68,"OK")</f>
         <v/>
       </c>
       <c r="E11" s="20">
@@ -3172,7 +3299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H138"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3305,7 +3432,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: a yellow tile anywhere rules out sea of green</t>
+          <t>AchievementBadgeTest: a retired region in an old save does not count toward world explorer</t>
         </is>
       </c>
       <c r="C4" s="26" t="inlineStr">
@@ -3342,7 +3469,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: a zero duration does not count as fast</t>
+          <t>AchievementBadgeTest: a yellow tile anywhere rules out sea of green</t>
         </is>
       </c>
       <c r="C5" s="26" t="inlineStr">
@@ -3379,7 +3506,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: achievements are awarded once</t>
+          <t>AchievementBadgeTest: a zero duration does not count as fast</t>
         </is>
       </c>
       <c r="C6" s="26" t="inlineStr">
@@ -3416,7 +3543,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: clean kitchen needs zero power-ups</t>
+          <t>AchievementBadgeTest: achievements are awarded once</t>
         </is>
       </c>
       <c r="C7" s="26" t="inlineStr">
@@ -3453,7 +3580,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: fast thinker is under the threshold</t>
+          <t>AchievementBadgeTest: clean kitchen needs zero power-ups</t>
         </is>
       </c>
       <c r="C8" s="26" t="inlineStr">
@@ -3490,7 +3617,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: instant solve cannot buy sea of green</t>
+          <t>AchievementBadgeTest: fast thinker is under the threshold</t>
         </is>
       </c>
       <c r="C9" s="26" t="inlineStr">
@@ -3527,7 +3654,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: instant solve does not count as a last plating</t>
+          <t>AchievementBadgeTest: instant solve cannot buy sea of green</t>
         </is>
       </c>
       <c r="C10" s="26" t="inlineStr">
@@ -3564,7 +3691,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: knowledge badges count distinct dishes read</t>
+          <t>AchievementBadgeTest: instant solve does not count as a last plating</t>
         </is>
       </c>
       <c r="C11" s="26" t="inlineStr">
@@ -3601,7 +3728,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: last plating is the final row only</t>
+          <t>AchievementBadgeTest: knowledge badges count distinct dishes read</t>
         </is>
       </c>
       <c r="C12" s="26" t="inlineStr">
@@ -3638,7 +3765,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: re-reading the same dish changes nothing</t>
+          <t>AchievementBadgeTest: last plating is the final row only</t>
         </is>
       </c>
       <c r="C13" s="26" t="inlineStr">
@@ -3675,7 +3802,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: replaying a solved dish cannot re-earn an achievement</t>
+          <t>AchievementBadgeTest: re-reading the same dish changes nothing</t>
         </is>
       </c>
       <c r="C14" s="26" t="inlineStr">
@@ -3712,7 +3839,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: sea of green needs no yellow and more than one guess</t>
+          <t>AchievementBadgeTest: replaying a solved dish cannot re-earn an achievement</t>
         </is>
       </c>
       <c r="C15" s="26" t="inlineStr">
@@ -3749,7 +3876,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: solving twice in one region does not count twice</t>
+          <t>AchievementBadgeTest: sea of green needs no yellow and more than one guess</t>
         </is>
       </c>
       <c r="C16" s="26" t="inlineStr">
@@ -3786,7 +3913,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>AchievementBadgeTest: world explorer needs every region</t>
+          <t>AchievementBadgeTest: solving twice in one region does not count twice</t>
         </is>
       </c>
       <c r="C17" s="26" t="inlineStr">
@@ -3823,7 +3950,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>BadgeArtTest: an unknown badge returns null rather than throwing</t>
+          <t>AchievementBadgeTest: world explorer needs every region</t>
         </is>
       </c>
       <c r="C18" s="26" t="inlineStr">
@@ -3860,7 +3987,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>BadgeArtTest: art is keyed on the badge id, not the title</t>
+          <t>BadgeArtTest: an unknown badge returns null rather than throwing</t>
         </is>
       </c>
       <c r="C19" s="26" t="inlineStr">
@@ -3897,7 +4024,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>BadgeArtTest: distinct badges get distinct medals</t>
+          <t>BadgeArtTest: art is keyed on the badge id, not the title</t>
         </is>
       </c>
       <c r="C20" s="26" t="inlineStr">
@@ -3934,7 +4061,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>BadgeArtTest: every badge in the catalogue has artwork</t>
+          <t>BadgeArtTest: distinct badges get distinct medals</t>
         </is>
       </c>
       <c r="C21" s="26" t="inlineStr">
@@ -3971,7 +4098,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>BadgeRulesTest: a badge already held is never awarded twice</t>
+          <t>BadgeArtTest: every badge in the catalogue has artwork</t>
         </is>
       </c>
       <c r="C22" s="26" t="inlineStr">
@@ -4008,7 +4135,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>BadgeRulesTest: catalog ids are unique</t>
+          <t>BadgeRulesTest: a badge already held is never awarded twice</t>
         </is>
       </c>
       <c r="C23" s="26" t="inlineStr">
@@ -4045,7 +4172,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>BadgeRulesTest: every badge family has at least one badge in the catalog</t>
+          <t>BadgeRulesTest: catalog ids are unique</t>
         </is>
       </c>
       <c r="C24" s="26" t="inlineStr">
@@ -4082,7 +4209,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>BadgeRulesTest: nothing is awarded before the first milestone</t>
+          <t>BadgeRulesTest: every badge family has at least one badge in the catalog</t>
         </is>
       </c>
       <c r="C25" s="26" t="inlineStr">
@@ -4119,7 +4246,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>BadgeRulesTest: passing a milestone unnoticed still awards it later</t>
+          <t>BadgeRulesTest: nothing is awarded before the first milestone</t>
         </is>
       </c>
       <c r="C26" s="26" t="inlineStr">
@@ -4156,7 +4283,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>BadgeRulesTest: perfect badges track first-guess solves</t>
+          <t>BadgeRulesTest: passing a milestone unnoticed still awards it later</t>
         </is>
       </c>
       <c r="C27" s="26" t="inlineStr">
@@ -4193,7 +4320,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>BadgeRulesTest: round badge fires exactly on the threshold, not before</t>
+          <t>BadgeRulesTest: perfect badges track first-guess solves</t>
         </is>
       </c>
       <c r="C28" s="26" t="inlineStr">
@@ -4230,7 +4357,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>BadgeRulesTest: streak badges follow the best streak, not the current one</t>
+          <t>BadgeRulesTest: round badge fires exactly on the threshold, not before</t>
         </is>
       </c>
       <c r="C29" s="26" t="inlineStr">
@@ -4267,7 +4394,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>BadgeRulesTest: the three families the manuscript names are all present</t>
+          <t>BadgeRulesTest: streak badges follow the best streak, not the current one</t>
         </is>
       </c>
       <c r="C30" s="26" t="inlineStr">
@@ -4304,7 +4431,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>EquipmentArtTest: an unknown tool returns null rather than throwing</t>
+          <t>BadgeRulesTest: the three families the manuscript names are all present</t>
         </is>
       </c>
       <c r="C31" s="26" t="inlineStr">
@@ -4341,7 +4468,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>EquipmentArtTest: every tool named in the dataset resolves to artwork</t>
+          <t>ChefRankTest: Head Chef leads to Kusina Master at the whole catalogue</t>
         </is>
       </c>
       <c r="C32" s="26" t="inlineStr">
@@ -4378,7 +4505,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>EquipmentArtTest: lookup ignores punctuation and casing differences in the sheet</t>
+          <t>ChefRankTest: a new player is a Kusinero heading for Line Cook</t>
         </is>
       </c>
       <c r="C33" s="26" t="inlineStr">
@@ -4415,7 +4542,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>ErrorMappingTest: a dropped socket is unreachable</t>
+          <t>ChefRankTest: a short catalogue skips steps it cannot reach</t>
         </is>
       </c>
       <c r="C34" s="26" t="inlineStr">
@@ -4452,7 +4579,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>ErrorMappingTest: a refused connection is unreachable, not unknown</t>
+          <t>ChefRankTest: every dish solved is Kusina Master, with nothing above it</t>
         </is>
       </c>
       <c r="C35" s="26" t="inlineStr">
@@ -4489,7 +4616,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>ErrorMappingTest: a server refusal keeps its own wording and hides technical noise</t>
+          <t>ChefRankTest: ranks change exactly at the round badge thresholds</t>
         </is>
       </c>
       <c r="C36" s="26" t="inlineStr">
@@ -4526,7 +4653,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>ErrorMappingTest: a successful result passes through untouched</t>
+          <t>ChefRankTest: the ladder lists every rank up to Kusina Master at the total</t>
         </is>
       </c>
       <c r="C37" s="26" t="inlineStr">
@@ -4563,7 +4690,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>ErrorMappingTest: a timeout reads as the server not answering, not as being offline</t>
+          <t>EquipmentArtTest: an unknown tool returns null rather than throwing</t>
         </is>
       </c>
       <c r="C38" s="26" t="inlineStr">
@@ -4600,7 +4727,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>ErrorMappingTest: an unrecognised failure still produces something calm and retryable</t>
+          <t>EquipmentArtTest: every tool named in the dataset resolves to artwork</t>
         </is>
       </c>
       <c r="C39" s="26" t="inlineStr">
@@ -4637,7 +4764,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>ErrorMappingTest: an unresolvable host reads as offline</t>
+          <t>EquipmentArtTest: lookup ignores punctuation and casing differences in the sheet</t>
         </is>
       </c>
       <c r="C40" s="26" t="inlineStr">
@@ -4674,7 +4801,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>ErrorMappingTest: mapNetworkError wraps a failure once, not repeatedly</t>
+          <t>ErrorMappingTest: a dropped socket is unreachable</t>
         </is>
       </c>
       <c r="C41" s="26" t="inlineStr">
@@ -4711,7 +4838,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>ErrorMappingTest: no message ever leaks a raw url into the headline</t>
+          <t>ErrorMappingTest: a refused connection is unreachable, not unknown</t>
         </is>
       </c>
       <c r="C42" s="26" t="inlineStr">
@@ -4748,7 +4875,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>ExampleUnitTest: addition_isCorrect</t>
+          <t>ErrorMappingTest: a server refusal keeps its own wording and hides technical noise</t>
         </is>
       </c>
       <c r="C43" s="26" t="inlineStr">
@@ -4785,7 +4912,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>FeaturedBadgesTest: a chosen badge that is not earned is dropped, not shown as locked</t>
+          <t>ErrorMappingTest: a successful result passes through untouched</t>
         </is>
       </c>
       <c r="C44" s="26" t="inlineStr">
@@ -4822,7 +4949,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>FeaturedBadgesTest: a chosen showcase is shown in the player's order</t>
+          <t>ErrorMappingTest: a timeout reads as the server not answering, not as being offline</t>
         </is>
       </c>
       <c r="C45" s="26" t="inlineStr">
@@ -4859,7 +4986,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>FeaturedBadgesTest: a new player with nothing earned still sees locked slots to aim at</t>
+          <t>ErrorMappingTest: an unrecognised failure still produces something calm and retryable</t>
         </is>
       </c>
       <c r="C46" s="26" t="inlineStr">
@@ -4896,7 +5023,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>FeaturedBadgesTest: a partial choice is topped up rather than leaving gaps</t>
+          <t>ErrorMappingTest: an unresolvable host reads as offline</t>
         </is>
       </c>
       <c r="C47" s="26" t="inlineStr">
@@ -4933,7 +5060,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>FeaturedBadgesTest: a short roster does not pad beyond what exists</t>
+          <t>ErrorMappingTest: mapNetworkError wraps a failure once, not repeatedly</t>
         </is>
       </c>
       <c r="C48" s="26" t="inlineStr">
@@ -4950,7 +5077,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>FeaturedBadgesTest: more choices than slots are trimmed to the first ones</t>
+          <t>ErrorMappingTest: no message ever leaks a raw url into the headline</t>
         </is>
       </c>
       <c r="C49" s="26" t="inlineStr">
@@ -4967,7 +5094,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>FeaturedBadgesTest: no choice falls back to earned badges first</t>
+          <t>ExampleUnitTest: addition_isCorrect</t>
         </is>
       </c>
       <c r="C50" s="26" t="inlineStr">
@@ -4984,7 +5111,7 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>FeaturedBadgesTest: the shelf never repeats a badge</t>
+          <t>FeaturedBadgesTest: a chosen badge that is not earned is dropped, not shown as locked</t>
         </is>
       </c>
       <c r="C51" s="26" t="inlineStr">
@@ -5001,7 +5128,7 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: a finished round is dropped rather than resumed</t>
+          <t>FeaturedBadgesTest: a chosen showcase is shown in the player's order</t>
         </is>
       </c>
       <c r="C52" s="26" t="inlineStr">
@@ -5018,7 +5145,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: a snapshot from a different word length is discarded</t>
+          <t>FeaturedBadgesTest: a new player with nothing earned still sees locked slots to aim at</t>
         </is>
       </c>
       <c r="C53" s="26" t="inlineStr">
@@ -5035,7 +5162,7 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: an untouched board is not treated as something to resume</t>
+          <t>FeaturedBadgesTest: a partial choice is topped up rather than leaving gaps</t>
         </is>
       </c>
       <c r="C54" s="26" t="inlineStr">
@@ -5052,7 +5179,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: attempt duration is reported in milliseconds</t>
+          <t>FeaturedBadgesTest: a short roster does not pad beyond what exists</t>
         </is>
       </c>
       <c r="C55" s="26" t="inlineStr">
@@ -5069,7 +5196,7 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: board is six rows tall regardless of word length</t>
+          <t>FeaturedBadgesTest: more choices than slots are trimmed to the first ones</t>
         </is>
       </c>
       <c r="C56" s="26" t="inlineStr">
@@ -5086,7 +5213,7 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: correct guess wins the round and completes the level</t>
+          <t>FeaturedBadgesTest: no choice falls back to earned badges first</t>
         </is>
       </c>
       <c r="C57" s="26" t="inlineStr">
@@ -5103,7 +5230,7 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: every submitted guess is recorded with level and correctness</t>
+          <t>FeaturedBadgesTest: the shelf never repeats a badge</t>
         </is>
       </c>
       <c r="C58" s="26" t="inlineStr">
@@ -5120,7 +5247,7 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: grid dimensions follow word length, not a fixed 6x6</t>
+          <t>GameViewModelTest: a finished round is dropped rather than resumed</t>
         </is>
       </c>
       <c r="C59" s="26" t="inlineStr">
@@ -5137,7 +5264,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: incomplete guess is not evaluated or recorded</t>
+          <t>GameViewModelTest: a snapshot from a different word length is discarded</t>
         </is>
       </c>
       <c r="C60" s="26" t="inlineStr">
@@ -5154,7 +5281,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: instant solve does nothing without enough KK</t>
+          <t>GameViewModelTest: an untouched board is not treated as something to resume</t>
         </is>
       </c>
       <c r="C61" s="26" t="inlineStr">
@@ -5171,7 +5298,7 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: instant solve fills the answer and ends the round</t>
+          <t>GameViewModelTest: attempt duration is reported in milliseconds</t>
         </is>
       </c>
       <c r="C62" s="26" t="inlineStr">
@@ -5188,7 +5315,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: leaving mid-round and coming back resumes the same board</t>
+          <t>GameViewModelTest: board is six rows tall regardless of word length</t>
         </is>
       </c>
       <c r="C63" s="26" t="inlineStr">
@@ -5205,7 +5332,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: no input accepted after the round ends</t>
+          <t>GameViewModelTest: correct guess wins the round and completes the level</t>
         </is>
       </c>
       <c r="C64" s="26" t="inlineStr">
@@ -5222,7 +5349,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: restart resets the round completely</t>
+          <t>GameViewModelTest: every submitted guess is recorded with level and correctness</t>
         </is>
       </c>
       <c r="C65" s="26" t="inlineStr">
@@ -5239,7 +5366,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: reveal does not lock a column already marked green</t>
+          <t>GameViewModelTest: grid dimensions follow word length, not a fixed 6x6</t>
         </is>
       </c>
       <c r="C66" s="26" t="inlineStr">
@@ -5256,7 +5383,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: reveal does not spend KK when every column is already green</t>
+          <t>GameViewModelTest: incomplete guess is not evaluated or recorded</t>
         </is>
       </c>
       <c r="C67" s="26" t="inlineStr">
@@ -5273,7 +5400,7 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: round ends in game over after max attempts of wrong guesses</t>
+          <t>GameViewModelTest: instant solve does nothing without enough KK</t>
         </is>
       </c>
       <c r="C68" s="26" t="inlineStr">
@@ -5290,7 +5417,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>GameViewModelTest: timer ticks only while unpaused and round is active</t>
+          <t>GameViewModelTest: instant solve fills the answer and ends the round</t>
         </is>
       </c>
       <c r="C69" s="26" t="inlineStr">
@@ -5307,7 +5434,7 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: a genuinely new level still scores after seeding</t>
+          <t>GameViewModelTest: leaving mid-round and coming back resumes the same board</t>
         </is>
       </c>
       <c r="C70" s="26" t="inlineStr">
@@ -5324,7 +5451,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: a power-up the player cannot afford charges nothing</t>
+          <t>GameViewModelTest: no input accepted after the round ends</t>
         </is>
       </c>
       <c r="C71" s="26" t="inlineStr">
@@ -5341,7 +5468,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: an account the server has never seen still bootstraps locally</t>
+          <t>GameViewModelTest: restart resets the round completely</t>
         </is>
       </c>
       <c r="C72" s="26" t="inlineStr">
@@ -5358,7 +5485,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: badges are awarded once even across repeated rounds</t>
+          <t>GameViewModelTest: reveal does not lock a column already marked green</t>
         </is>
       </c>
       <c r="C73" s="26" t="inlineStr">
@@ -5375,7 +5502,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: dishes solved before gamification existed are credited once</t>
+          <t>GameViewModelTest: reveal does not spend KK when every column is already green</t>
         </is>
       </c>
       <c r="C74" s="26" t="inlineStr">
@@ -5392,7 +5519,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: points spent on a power-up are not handed back by the next sync</t>
+          <t>GameViewModelTest: round ends in game over after max attempts of wrong guesses</t>
         </is>
       </c>
       <c r="C75" s="26" t="inlineStr">
@@ -5409,7 +5536,7 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: replaying the same level does not award points twice</t>
+          <t>GameViewModelTest: timer ticks only while unpaused and round is active</t>
         </is>
       </c>
       <c r="C76" s="26" t="inlineStr">
@@ -5426,7 +5553,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: restored solved levels still block replay farming</t>
+          <t>GamificationCoordinatorTest: a genuinely new level still scores after seeding</t>
         </is>
       </c>
       <c r="C77" s="26" t="inlineStr">
@@ -5443,7 +5570,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: seeding grants the badges those old solves already earned</t>
+          <t>GamificationCoordinatorTest: a power-up the player cannot afford charges nothing</t>
         </is>
       </c>
       <c r="C78" s="26" t="inlineStr">
@@ -5460,7 +5587,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>GamificationCoordinatorTest: signing in on a new device restores the account's real state</t>
+          <t>GamificationCoordinatorTest: an account the server has never seen still bootstraps locally</t>
         </is>
       </c>
       <c r="C79" s="26" t="inlineStr">
@@ -5477,7 +5604,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>IngredientArtTest: an unknown ingredient returns null rather than throwing</t>
+          <t>GamificationCoordinatorTest: badges are awarded once even across repeated rounds</t>
         </is>
       </c>
       <c r="C80" s="26" t="inlineStr">
@@ -5494,7 +5621,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>IngredientArtTest: coverage is real, not an empty dataset</t>
+          <t>GamificationCoordinatorTest: dishes solved before gamification existed are credited once</t>
         </is>
       </c>
       <c r="C81" s="26" t="inlineStr">
@@ -5511,7 +5638,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>IngredientArtTest: every ingredient in the dataset has photography</t>
+          <t>GamificationCoordinatorTest: points spent on a power-up are not handed back by the next sync</t>
         </is>
       </c>
       <c r="C82" s="26" t="inlineStr">
@@ -5528,7 +5655,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>IngredientArtTest: lookup ignores casing and punctuation</t>
+          <t>GamificationCoordinatorTest: replaying the same level does not award points twice</t>
         </is>
       </c>
       <c r="C83" s="26" t="inlineStr">
@@ -5545,7 +5672,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>IngredientLineTest: bare measurements are dropped</t>
+          <t>GamificationCoordinatorTest: restored solved levels still block replay farming</t>
         </is>
       </c>
       <c r="C84" s="26" t="inlineStr">
@@ -5562,7 +5689,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>IngredientLineTest: duplicates are removed, keeping the first spelling</t>
+          <t>GamificationCoordinatorTest: seeding grants the badges those old solves already earned</t>
         </is>
       </c>
       <c r="C85" s="26" t="inlineStr">
@@ -5579,7 +5706,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>IngredientLineTest: headers and measurements are stripped from the whole list</t>
+          <t>GamificationCoordinatorTest: signing in on a new device restores the account's real state</t>
         </is>
       </c>
       <c r="C86" s="26" t="inlineStr">
@@ -5596,7 +5723,7 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>IngredientLineTest: matching ignores case and surrounding space</t>
+          <t>HeldLevelsTest: Piaya is Visayas Level 3</t>
         </is>
       </c>
       <c r="C87" s="26" t="inlineStr">
@@ -5613,7 +5740,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>IngredientLineTest: only the first word is read as a unit</t>
+          <t>HeldLevelsTest: Piaya, Kulma and Pigar-Pigar are levels 28 to 30, the web panel's ids</t>
         </is>
       </c>
       <c r="C88" s="26" t="inlineStr">
@@ -5630,7 +5757,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>IngredientLineTest: real ingredients are kept</t>
+          <t>HeldLevelsTest: a Draft on a normal level does not hide it</t>
         </is>
       </c>
       <c r="C89" s="26" t="inlineStr">
@@ -5647,7 +5774,7 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>IngredientLineTest: section headers are dropped</t>
+          <t>HeldLevelsTest: held levels start hidden until the panel publishes them</t>
         </is>
       </c>
       <c r="C90" s="26" t="inlineStr">
@@ -5664,7 +5791,7 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>IngredientLineTest: sheet order is preserved</t>
+          <t>HeldLevelsTest: hidden levels are left out of the island order and the counts</t>
         </is>
       </c>
       <c r="C91" s="26" t="inlineStr">
@@ -5681,7 +5808,7 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>IngredientLineTest: stray values and blanks are dropped</t>
+          <t>HeldLevelsTest: once published, each held dish is the last of its island</t>
         </is>
       </c>
       <c r="C92" s="26" t="inlineStr">
@@ -5698,7 +5825,7 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>IslandRulesTest: an island pays only when every dish there is solved</t>
+          <t>HeldLevelsTest: publishing shows a held level and Draft hides it again, numbers unchanged</t>
         </is>
       </c>
       <c r="C93" s="26" t="inlineStr">
@@ -5715,7 +5842,7 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>KusinaShopTest: learning content stays cheap and cosmetics are the premium tier</t>
+          <t>HeldLevelsTest: the board shows a dash only where the name has one</t>
         </is>
       </c>
       <c r="C94" s="26" t="inlineStr">
@@ -5732,7 +5859,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>LeaderboardRulesTest: an empty board ranks to nothing rather than failing</t>
+          <t>HeldLevelsTest: the first 27 level numbers are exactly as they shipped</t>
         </is>
       </c>
       <c r="C95" s="26" t="inlineStr">
@@ -5749,7 +5876,7 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>LeaderboardRulesTest: dishes solved break a points tie</t>
+          <t>HeldLevelsTest: the panel may write Pigar-Pigar with its hyphen</t>
         </is>
       </c>
       <c r="C96" s="26" t="inlineStr">
@@ -5766,7 +5893,7 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>LeaderboardRulesTest: earning points moves a player up the board</t>
+          <t>IngredientArtTest: an unknown ingredient returns null rather than throwing</t>
         </is>
       </c>
       <c r="C97" s="26" t="inlineStr">
@@ -5783,7 +5910,7 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>LeaderboardRulesTest: name breaks a full tie so the order never shuffles</t>
+          <t>IngredientArtTest: coverage is real, not an empty dataset</t>
         </is>
       </c>
       <c r="C98" s="26" t="inlineStr">
@@ -5800,7 +5927,7 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>LeaderboardRulesTest: players are ordered by points, highest first</t>
+          <t>IngredientArtTest: every ingredient in the book has a picture by its name</t>
         </is>
       </c>
       <c r="C99" s="26" t="inlineStr">
@@ -5817,7 +5944,7 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>LeaderboardRulesTest: players yet to score still appear, at the bottom</t>
+          <t>IngredientArtTest: every ingredient in the dataset has photography</t>
         </is>
       </c>
       <c r="C100" s="26" t="inlineStr">
@@ -5834,7 +5961,7 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>LeaderboardRulesTest: position lookup ignores case and reports absence</t>
+          <t>IngredientArtTest: lookup ignores casing and punctuation</t>
         </is>
       </c>
       <c r="C101" s="26" t="inlineStr">
@@ -5851,7 +5978,7 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>PalayokGrantRulesTest: a win pays one palayok</t>
+          <t>IngredientArtTest: the web console's names get the pantry picture</t>
         </is>
       </c>
       <c r="C102" s="26" t="inlineStr">
@@ -5868,7 +5995,7 @@
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>PalayokGrantRulesTest: nothing is held back for the pantry shelf</t>
+          <t>IngredientCatalogRemoteTest: a new web ingredient joins the book after the bundled ones</t>
         </is>
       </c>
       <c r="C103" s="26" t="inlineStr">
@@ -5885,7 +6012,7 @@
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>PantryIngredientArtTest: an unknown id returns null rather than throwing</t>
+          <t>IngredientCatalogRemoteTest: an empty web list keeps the bundled book</t>
         </is>
       </c>
       <c r="C104" s="26" t="inlineStr">
@@ -5902,7 +6029,7 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>PantryIngredientArtTest: coverage is real, not an empty catalog</t>
+          <t>IngredientCatalogRemoteTest: an id no list knows still resolves, so a jar is never dropped</t>
         </is>
       </c>
       <c r="C105" s="26" t="inlineStr">
@@ -5919,7 +6046,7 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>PantryIngredientArtTest: every catalog ingredient has a photo</t>
+          <t>IngredientCatalogRemoteTest: an ingredient the web no longer lists leaves the book but stays nameable</t>
         </is>
       </c>
       <c r="C106" s="26" t="inlineStr">
@@ -5936,7 +6063,7 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>PowerUpRulesTest: a nearly exhausted keyboard bombs nothing rather than misbehaving</t>
+          <t>IngredientCatalogRemoteTest: an unknown rarity reads as common</t>
         </is>
       </c>
       <c r="C107" s="26" t="inlineStr">
@@ -5953,7 +6080,7 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>PowerUpRulesTest: a second hint waits one minute</t>
+          <t>IngredientCatalogRemoteTest: the web's wording and rarity win for a known id</t>
         </is>
       </c>
       <c r="C108" s="26" t="inlineStr">
@@ -5970,7 +6097,7 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>PowerUpRulesTest: bomb leaves the agreed number of decoys standing</t>
+          <t>IngredientCatalogRemoteTest: with nothing from the web the bundled book stands</t>
         </is>
       </c>
       <c r="C109" s="26" t="inlineStr">
@@ -5987,7 +6114,7 @@
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>PowerUpRulesTest: bomb never clears a letter that is in the answer</t>
+          <t>IngredientLineTest: bare measurements are dropped</t>
         </is>
       </c>
       <c r="C110" s="26" t="inlineStr">
@@ -6004,7 +6131,7 @@
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>PowerUpRulesTest: letters already ruled out are not counted again</t>
+          <t>IngredientLineTest: duplicates are removed, keeping the first spelling</t>
         </is>
       </c>
       <c r="C111" s="26" t="inlineStr">
@@ -6021,7 +6148,7 @@
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>PowerUpRulesTest: reveal and bomb are KK-priced, never XP</t>
+          <t>IngredientLineTest: headers and measurements are stripped from the whole list</t>
         </is>
       </c>
       <c r="C112" s="26" t="inlineStr">
@@ -6038,7 +6165,7 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>ProgressRulesTest: a loss resets the streak but keeps points and best streak</t>
+          <t>IngredientLineTest: matching ignores case and surrounding space</t>
         </is>
       </c>
       <c r="C113" s="26" t="inlineStr">
@@ -6055,7 +6182,7 @@
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>ProgressRulesTest: a win adds points and advances every counter</t>
+          <t>IngredientLineTest: only the first word is read as a unit</t>
         </is>
       </c>
       <c r="C114" s="26" t="inlineStr">
@@ -6072,7 +6199,7 @@
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>ProgressRulesTest: best streak survives a later break</t>
+          <t>IngredientLineTest: real ingredients are kept</t>
         </is>
       </c>
       <c r="C115" s="26" t="inlineStr">
@@ -6089,7 +6216,7 @@
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>ProgressRulesTest: perfect rounds are counted separately</t>
+          <t>IngredientLineTest: section headers are dropped</t>
         </is>
       </c>
       <c r="C116" s="26" t="inlineStr">
@@ -6106,7 +6233,7 @@
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>ProgressRulesTest: points accumulate across separate rounds</t>
+          <t>IngredientLineTest: sheet order is preserved</t>
         </is>
       </c>
       <c r="C117" s="26" t="inlineStr">
@@ -6123,7 +6250,7 @@
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>ProgressRulesTest: replaying a solved dish scores nothing</t>
+          <t>IngredientLineTest: stray values and blanks are dropped</t>
         </is>
       </c>
       <c r="C118" s="26" t="inlineStr">
@@ -6140,7 +6267,7 @@
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>ReportDetailsTest: a real sentence is accepted</t>
+          <t>IslandRulesTest: an island pays only when every dish there is solved</t>
         </is>
       </c>
       <c r="C119" s="26" t="inlineStr">
@@ -6157,7 +6284,7 @@
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>ReportDetailsTest: aaa is rejected as not a real description</t>
+          <t>KusinaShopTest: learning content stays cheap and cosmetics are the premium tier</t>
         </is>
       </c>
       <c r="C120" s="26" t="inlineStr">
@@ -6174,7 +6301,7 @@
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>ReportDetailsTest: blank is rejected</t>
+          <t>LeaderboardRulesTest: an empty board ranks to nothing rather than failing</t>
         </is>
       </c>
       <c r="C121" s="26" t="inlineStr">
@@ -6191,7 +6318,7 @@
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>ScoreRulesTest: first-guess solve earns the perfect bonus</t>
+          <t>LeaderboardRulesTest: dishes solved break a points tie</t>
         </is>
       </c>
       <c r="C122" s="26" t="inlineStr">
@@ -6208,7 +6335,7 @@
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>ScoreRulesTest: identical rounds always score identically</t>
+          <t>LeaderboardRulesTest: earning points moves a player up the board</t>
         </is>
       </c>
       <c r="C123" s="26" t="inlineStr">
@@ -6225,7 +6352,7 @@
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>ScoreRulesTest: overrunning the allowance never subtracts points</t>
+          <t>LeaderboardRulesTest: name breaks a full tie so the order never shuffles</t>
         </is>
       </c>
       <c r="C124" s="26" t="inlineStr">
@@ -6242,7 +6369,7 @@
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>ScoreRulesTest: solving on the last attempt still scores the base award</t>
+          <t>LeaderboardRulesTest: players are ordered by points, highest first</t>
         </is>
       </c>
       <c r="C125" s="26" t="inlineStr">
@@ -6259,7 +6386,7 @@
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>ScoreRulesTest: speed bonus follows its tiers</t>
+          <t>LeaderboardRulesTest: players yet to score still appear, at the bottom</t>
         </is>
       </c>
       <c r="C126" s="26" t="inlineStr">
@@ -6276,7 +6403,7 @@
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>ScoreRulesTest: tier boundaries are exclusive at the upper edge</t>
+          <t>LeaderboardRulesTest: position lookup ignores case and reports absence</t>
         </is>
       </c>
       <c r="C127" s="26" t="inlineStr">
@@ -6293,7 +6420,7 @@
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>ScoreRulesTest: unused attempts add efficiency points</t>
+          <t>LeaderboardViewModelTest: playerOutsideTopTen_keepsTheirOwnRank</t>
         </is>
       </c>
       <c r="C128" s="26" t="inlineStr">
@@ -6310,7 +6437,7 @@
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>WordleEngineTest: all letters correct when guess equals answer, case-insensitive</t>
+          <t>LeaderboardViewModelTest: signedOut_hasNoStanding</t>
         </is>
       </c>
       <c r="C129" s="26" t="inlineStr">
@@ -6327,7 +6454,7 @@
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>WordleEngineTest: complete alphabetic guess is valid at 5, 6 and 8 letters</t>
+          <t>LeaderboardViewModelTest: switchingBoards_dropsTheOldStanding</t>
         </is>
       </c>
       <c r="C130" s="26" t="inlineStr">
@@ -6344,7 +6471,7 @@
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>WordleEngineTest: evaluate rejects mismatched guess length</t>
+          <t>LevelOrderPinsTest: Kinilaw added with no pin goes by its length</t>
         </is>
       </c>
       <c r="C131" s="26" t="inlineStr">
@@ -6361,7 +6488,7 @@
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>WordleEngineTest: evaluate works for 8-letter words</t>
+          <t>LevelOrderPinsTest: Kinilaw pinned to 2 takes Level 2</t>
         </is>
       </c>
       <c r="C132" s="26" t="inlineStr">
@@ -6378,7 +6505,7 @@
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>WordleEngineTest: every word length gets six attempts</t>
+          <t>LevelOrderPinsTest: Luzon with Sisig pinned to 2</t>
         </is>
       </c>
       <c r="C133" s="26" t="inlineStr">
@@ -6395,7 +6522,7 @@
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>WordleEngineTest: incomplete guess is rejected for any word length</t>
+          <t>LevelOrderPinsTest: Mindanao today, no pins</t>
         </is>
       </c>
       <c r="C134" s="26" t="inlineStr">
@@ -6412,7 +6539,7 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>WordleEngineTest: misplaced repeated letters consume answer occurrences left to right</t>
+          <t>LevelOrderPinsTest: Satti pinned to 6 and Tiyula to 1</t>
         </is>
       </c>
       <c r="C135" s="26" t="inlineStr">
@@ -6429,7 +6556,7 @@
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>WordleEngineTest: mixed verdict classifies correct, misplaced and absent letters</t>
+          <t>LevelOrderPinsTest: a pin only reads as a whole number of 1 or more</t>
         </is>
       </c>
       <c r="C136" s="26" t="inlineStr">
@@ -6446,7 +6573,7 @@
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>WordleEngineTest: non-letter characters are rejected</t>
+          <t>LevelOrderPinsTest: a pin past the end counts as the last slot</t>
         </is>
       </c>
       <c r="C137" s="26" t="inlineStr">
@@ -6463,10 +6590,1013 @@
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
+          <t>LevelOrderPinsTest: the Game Map's next level follows a pin</t>
+        </is>
+      </c>
+      <c r="C138" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="19" t="inlineStr">
+        <is>
+          <t>U-138</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>LevelOrderPinsTest: two pins on one slot, the lower id keeps it</t>
+        </is>
+      </c>
+      <c r="C139" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="19" t="inlineStr">
+        <is>
+          <t>U-139</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>LevelOrderPinsTest: two pins on the last slot, the second takes the nearest free one before it</t>
+        </is>
+      </c>
+      <c r="C140" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="19" t="inlineStr">
+        <is>
+          <t>U-140</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>PalayokGrantRulesTest: a win pays one palayok</t>
+        </is>
+      </c>
+      <c r="C141" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="19" t="inlineStr">
+        <is>
+          <t>U-141</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>PalayokGrantRulesTest: nothing is held back for the pantry shelf</t>
+        </is>
+      </c>
+      <c r="C142" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="19" t="inlineStr">
+        <is>
+          <t>U-142</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>PantryIngredientArtTest: an unknown id returns null rather than throwing</t>
+        </is>
+      </c>
+      <c r="C143" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="19" t="inlineStr">
+        <is>
+          <t>U-143</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>PantryIngredientArtTest: coverage is real, not an empty catalog</t>
+        </is>
+      </c>
+      <c r="C144" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="19" t="inlineStr">
+        <is>
+          <t>U-144</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>PantryIngredientArtTest: every catalog ingredient has a photo</t>
+        </is>
+      </c>
+      <c r="C145" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="19" t="inlineStr">
+        <is>
+          <t>U-145</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>PowerUpRulesTest: a nearly exhausted keyboard bombs nothing rather than misbehaving</t>
+        </is>
+      </c>
+      <c r="C146" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="19" t="inlineStr">
+        <is>
+          <t>U-146</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>PowerUpRulesTest: a second hint waits one minute</t>
+        </is>
+      </c>
+      <c r="C147" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="19" t="inlineStr">
+        <is>
+          <t>U-147</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>PowerUpRulesTest: bomb leaves the agreed number of decoys standing</t>
+        </is>
+      </c>
+      <c r="C148" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="19" t="inlineStr">
+        <is>
+          <t>U-148</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>PowerUpRulesTest: bomb never clears a letter that is in the answer</t>
+        </is>
+      </c>
+      <c r="C149" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="19" t="inlineStr">
+        <is>
+          <t>U-149</t>
+        </is>
+      </c>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t>PowerUpRulesTest: letters already ruled out are not counted again</t>
+        </is>
+      </c>
+      <c r="C150" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="19" t="inlineStr">
+        <is>
+          <t>U-150</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>PowerUpRulesTest: reveal and bomb are KK-priced, never XP</t>
+        </is>
+      </c>
+      <c r="C151" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="19" t="inlineStr">
+        <is>
+          <t>U-151</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>ProgressRulesTest: a loss resets the streak but keeps points and best streak</t>
+        </is>
+      </c>
+      <c r="C152" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="19" t="inlineStr">
+        <is>
+          <t>U-152</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>ProgressRulesTest: a win adds points and advances every counter</t>
+        </is>
+      </c>
+      <c r="C153" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="19" t="inlineStr">
+        <is>
+          <t>U-153</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>ProgressRulesTest: best streak survives a later break</t>
+        </is>
+      </c>
+      <c r="C154" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="19" t="inlineStr">
+        <is>
+          <t>U-154</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>ProgressRulesTest: perfect rounds are counted separately</t>
+        </is>
+      </c>
+      <c r="C155" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="19" t="inlineStr">
+        <is>
+          <t>U-155</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>ProgressRulesTest: points accumulate across separate rounds</t>
+        </is>
+      </c>
+      <c r="C156" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="19" t="inlineStr">
+        <is>
+          <t>U-156</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>ProgressRulesTest: replaying a solved dish scores nothing</t>
+        </is>
+      </c>
+      <c r="C157" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="19" t="inlineStr">
+        <is>
+          <t>U-157</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: a reel the admin adds appears on the shelf</t>
+        </is>
+      </c>
+      <c r="C158" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="19" t="inlineStr">
+        <is>
+          <t>U-158</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: a reel the admin withdraws leaves the shelf but still resolves</t>
+        </is>
+      </c>
+      <c r="C159" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="19" t="inlineStr">
+        <is>
+          <t>U-159</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: an empty response falls back to the seeds</t>
+        </is>
+      </c>
+      <c r="C160" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="19" t="inlineStr">
+        <is>
+          <t>U-160</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: an id the server never mentions keeps answering</t>
+        </is>
+      </c>
+      <c r="C161" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="19" t="inlineStr">
+        <is>
+          <t>U-161</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: every seeded reel has a price</t>
+        </is>
+      </c>
+      <c r="C162" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="19" t="inlineStr">
+        <is>
+          <t>U-162</t>
+        </is>
+      </c>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: ids stay unique after a merge</t>
+        </is>
+      </c>
+      <c r="C163" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="19" t="inlineStr">
+        <is>
+          <t>U-163</t>
+        </is>
+      </c>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: no overlay leaves the seeded shelf exactly as it was</t>
+        </is>
+      </c>
+      <c r="C164" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="19" t="inlineStr">
+        <is>
+          <t>U-164</t>
+        </is>
+      </c>
+      <c r="B165" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: non-reel items are untouched by the overlay</t>
+        </is>
+      </c>
+      <c r="C165" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="19" t="inlineStr">
+        <is>
+          <t>U-165</t>
+        </is>
+      </c>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: retired reels stay off the shelf but keep resolving</t>
+        </is>
+      </c>
+      <c r="C166" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="19" t="inlineStr">
+        <is>
+          <t>U-166</t>
+        </is>
+      </c>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: seed order survives a fetch</t>
+        </is>
+      </c>
+      <c r="C167" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="19" t="inlineStr">
+        <is>
+          <t>U-167</t>
+        </is>
+      </c>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>ReelCatalogTest: server wording and price win over the seed</t>
+        </is>
+      </c>
+      <c r="C168" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="19" t="inlineStr">
+        <is>
+          <t>U-168</t>
+        </is>
+      </c>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t>ReportDetailsTest: a real sentence is accepted</t>
+        </is>
+      </c>
+      <c r="C169" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="19" t="inlineStr">
+        <is>
+          <t>U-169</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>ReportDetailsTest: aaa is rejected as not a real description</t>
+        </is>
+      </c>
+      <c r="C170" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="19" t="inlineStr">
+        <is>
+          <t>U-170</t>
+        </is>
+      </c>
+      <c r="B171" s="4" t="inlineStr">
+        <is>
+          <t>ReportDetailsTest: blank is rejected</t>
+        </is>
+      </c>
+      <c r="C171" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="19" t="inlineStr">
+        <is>
+          <t>U-171</t>
+        </is>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t>ScoreRulesTest: first-guess solve earns the perfect bonus</t>
+        </is>
+      </c>
+      <c r="C172" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="19" t="inlineStr">
+        <is>
+          <t>U-172</t>
+        </is>
+      </c>
+      <c r="B173" s="4" t="inlineStr">
+        <is>
+          <t>ScoreRulesTest: identical rounds always score identically</t>
+        </is>
+      </c>
+      <c r="C173" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="19" t="inlineStr">
+        <is>
+          <t>U-173</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>ScoreRulesTest: overrunning the allowance never subtracts points</t>
+        </is>
+      </c>
+      <c r="C174" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="19" t="inlineStr">
+        <is>
+          <t>U-174</t>
+        </is>
+      </c>
+      <c r="B175" s="4" t="inlineStr">
+        <is>
+          <t>ScoreRulesTest: solving on the last attempt still scores the base award</t>
+        </is>
+      </c>
+      <c r="C175" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="19" t="inlineStr">
+        <is>
+          <t>U-175</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>ScoreRulesTest: speed bonus follows its tiers</t>
+        </is>
+      </c>
+      <c r="C176" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="19" t="inlineStr">
+        <is>
+          <t>U-176</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
+        <is>
+          <t>ScoreRulesTest: tier boundaries are exclusive at the upper edge</t>
+        </is>
+      </c>
+      <c r="C177" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="19" t="inlineStr">
+        <is>
+          <t>U-177</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>ScoreRulesTest: unused attempts add efficiency points</t>
+        </is>
+      </c>
+      <c r="C178" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="19" t="inlineStr">
+        <is>
+          <t>U-178</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t>SellAskTest: a chosen count sells only that many</t>
+        </is>
+      </c>
+      <c r="C179" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="19" t="inlineStr">
+        <is>
+          <t>U-179</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>SellAskTest: a single copy still sells one</t>
+        </is>
+      </c>
+      <c r="C180" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="19" t="inlineStr">
+        <is>
+          <t>U-180</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>SellAskTest: the count cannot pass the stack or drop below one</t>
+        </is>
+      </c>
+      <c r="C181" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="19" t="inlineStr">
+        <is>
+          <t>U-181</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>WaitingForYouCountTest: claimed daily with a leftover spin is one waiting row</t>
+        </is>
+      </c>
+      <c r="C182" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="19" t="inlineStr">
+        <is>
+          <t>U-182</t>
+        </is>
+      </c>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>WaitingForYouCountTest: history names a palayok spin without using the server key</t>
+        </is>
+      </c>
+      <c r="C183" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="19" t="inlineStr">
+        <is>
+          <t>U-183</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>WaitingForYouCountTest: nothing waiting is zero</t>
+        </is>
+      </c>
+      <c r="C184" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="19" t="inlineStr">
+        <is>
+          <t>U-184</t>
+        </is>
+      </c>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t>WaitingForYouCountTest: spin title carries the palayoks won</t>
+        </is>
+      </c>
+      <c r="C185" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="19" t="inlineStr">
+        <is>
+          <t>U-185</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>WaitingForYouCountTest: unclaimed daily is two rows even if a spin is already banked</t>
+        </is>
+      </c>
+      <c r="C186" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="19" t="inlineStr">
+        <is>
+          <t>U-186</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>WaitingForYouCountTest: unopened palayoks are one waiting row however many there are</t>
+        </is>
+      </c>
+      <c r="C187" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="19" t="inlineStr">
+        <is>
+          <t>U-187</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>WordleEngineTest: all letters correct when guess equals answer, case-insensitive</t>
+        </is>
+      </c>
+      <c r="C188" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="19" t="inlineStr">
+        <is>
+          <t>U-188</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>WordleEngineTest: complete alphabetic guess is valid at 5, 6 and 8 letters</t>
+        </is>
+      </c>
+      <c r="C189" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="19" t="inlineStr">
+        <is>
+          <t>U-189</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>WordleEngineTest: evaluate rejects mismatched guess length</t>
+        </is>
+      </c>
+      <c r="C190" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="19" t="inlineStr">
+        <is>
+          <t>U-190</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>WordleEngineTest: evaluate works for 8-letter words</t>
+        </is>
+      </c>
+      <c r="C191" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="19" t="inlineStr">
+        <is>
+          <t>U-191</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>WordleEngineTest: every word length gets six attempts</t>
+        </is>
+      </c>
+      <c r="C192" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="19" t="inlineStr">
+        <is>
+          <t>U-192</t>
+        </is>
+      </c>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t>WordleEngineTest: incomplete guess is rejected for any word length</t>
+        </is>
+      </c>
+      <c r="C193" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="19" t="inlineStr">
+        <is>
+          <t>U-193</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>WordleEngineTest: misplaced repeated letters consume answer occurrences left to right</t>
+        </is>
+      </c>
+      <c r="C194" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="19" t="inlineStr">
+        <is>
+          <t>U-194</t>
+        </is>
+      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t>WordleEngineTest: mixed verdict classifies correct, misplaced and absent letters</t>
+        </is>
+      </c>
+      <c r="C195" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="19" t="inlineStr">
+        <is>
+          <t>U-195</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>WordleEngineTest: non-letter characters are rejected</t>
+        </is>
+      </c>
+      <c r="C196" s="26" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="19" t="inlineStr">
+        <is>
+          <t>U-196</t>
+        </is>
+      </c>
+      <c r="B197" s="4" t="inlineStr">
+        <is>
           <t>WordleEngineTest: repeated guess letter is not flagged more times than it appears in answer</t>
         </is>
       </c>
-      <c r="C138" s="26" t="inlineStr">
+      <c r="C197" s="26" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>

</xml_diff>